<commit_message>
feat: add static publishing and protected vendor contacts
</commit_message>
<xml_diff>
--- a/docs/农机配件平台_厂商产品资料采集模板_河北春耕机械_最新版.xlsx
+++ b/docs/农机配件平台_厂商产品资料采集模板_河北春耕机械_最新版.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9180" activeTab="2"/>
+    <workbookView windowWidth="22188" windowHeight="9180" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="填写说明" sheetId="2" r:id="rId1"/>
@@ -1139,129 +1139,6 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1257300</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2" descr="DvYWao"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="19050" y="19050"/>
-          <a:ext cx="1238250" cy="403225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1257300</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>393700</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2" descr="bQdIGg"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="19050" y="19050"/>
-          <a:ext cx="1238250" cy="374650"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1257300</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 2" descr="UQwfGR"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="19050" y="19050"/>
-          <a:ext cx="1238250" cy="403225"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -1652,7 +1529,6 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1893,7 +1769,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2093,7 +1968,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>